<commit_message>
[T15583] 02:30 Incorpora nuevos cambios solicitados 12/8. Cambia posicion menuitem, contempla registrar facturas, contempla cae e impuestos.
</commit_message>
<xml_diff>
--- a/ivess_invoice_import/prueba_import_facturas.xlsx
+++ b/ivess_invoice_import/prueba_import_facturas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facturas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="facturas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:X12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,7 +619,6 @@
           <t>19000.00</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
       <c r="X2" t="n">
         <v>0</v>
       </c>
@@ -705,7 +704,6 @@
           <t>6200.00</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
       <c r="X3" t="n">
         <v>0</v>
       </c>
@@ -791,7 +789,6 @@
           <t>17500.00</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
       <c r="X4" t="n">
         <v>0</v>
       </c>
@@ -877,7 +874,6 @@
           <t>14700.00</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
       <c r="X5" t="n">
         <v>0</v>
       </c>
@@ -963,7 +959,6 @@
           <t>3280.00</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
       <c r="X6" t="n">
         <v>0</v>
       </c>
@@ -1049,7 +1044,6 @@
           <t>18300.00</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr"/>
       <c r="X7" t="n">
         <v>0</v>
       </c>
@@ -1135,9 +1129,368 @@
           <t>4750.00</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr"/>
       <c r="X8" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>900006</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20260727</v>
+      </c>
+      <c r="F9" t="n">
+        <v>500001</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ABELSON S.A.</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>30652000076</v>
+      </c>
+      <c r="I9" t="n">
+        <v>20260806</v>
+      </c>
+      <c r="J9" t="n">
+        <v>11995</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2000002N</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>10</v>
+      </c>
+      <c r="P9" t="n">
+        <v>950</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>21</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>1995</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>9500</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>9500.00</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>PERC_IIBB_CABA</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D10" t="n">
+        <v>900007</v>
+      </c>
+      <c r="E10" t="n">
+        <v>20260727</v>
+      </c>
+      <c r="F10" t="n">
+        <v>500001</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ABELSON S.A.</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>30652000076</v>
+      </c>
+      <c r="I10" t="n">
+        <v>20260806</v>
+      </c>
+      <c r="J10" t="n">
+        <v>11945</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2000002N</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>10</v>
+      </c>
+      <c r="P10" t="n">
+        <v>950</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>21</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1995</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>9500</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>9500.00</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>PERC_IIBB_ARBA</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>900008</v>
+      </c>
+      <c r="E11" t="n">
+        <v>20260727</v>
+      </c>
+      <c r="F11" t="n">
+        <v>500001</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ABELSON S.A.</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>30652000076</v>
+      </c>
+      <c r="I11" t="n">
+        <v>20260806</v>
+      </c>
+      <c r="J11" t="n">
+        <v>11795</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2000002N</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>10</v>
+      </c>
+      <c r="P11" t="n">
+        <v>950</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>21</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1995</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>9500</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>9500.00</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>PERC_IVA</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D12" t="n">
+        <v>900009</v>
+      </c>
+      <c r="E12" t="n">
+        <v>20260727</v>
+      </c>
+      <c r="F12" t="n">
+        <v>500001</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ABELSON S.A.</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>30652000076</v>
+      </c>
+      <c r="I12" t="n">
+        <v>20260806</v>
+      </c>
+      <c r="J12" t="n">
+        <v>12295</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2000002N</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>10</v>
+      </c>
+      <c r="P12" t="n">
+        <v>950</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>21</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="n">
+        <v>1995</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>9500</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>9500.00</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>IMP_INTERNO</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[T15583] 01:30 Agrega percepciones en excel para que lea y matchee en odoo, agrega contemplacion de nc y nd
</commit_message>
<xml_diff>
--- a/ivess_invoice_import/prueba_import_facturas.xlsx
+++ b/ivess_invoice_import/prueba_import_facturas.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="47">
   <si>
     <t xml:space="preserve">tipo de comprobante</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t xml:space="preserve">18300.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ND</t>
   </si>
   <si>
     <t xml:space="preserve">AVALOS BODDA SA</t>
@@ -274,7 +277,12 @@
   <dimension ref="A1:X11"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="29.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="19.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -359,10 +367,10 @@
         <v>25</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>900001</v>
+        <v>900007</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>20260727</v>
@@ -422,7 +430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -430,10 +438,10 @@
         <v>25</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>900001</v>
+        <v>900007</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>20260727</v>
@@ -493,7 +501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
@@ -501,10 +509,10 @@
         <v>25</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>900002</v>
+        <v>900008</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>20260727</v>
@@ -564,7 +572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -572,10 +580,10 @@
         <v>25</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>900003</v>
+        <v>900009</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>20260727</v>
@@ -635,7 +643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -643,10 +651,10 @@
         <v>25</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>900003</v>
+        <v>900009</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>20260727</v>
@@ -706,7 +714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
@@ -714,10 +722,10 @@
         <v>25</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>900004</v>
+        <v>900010</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>20260727</v>
@@ -777,18 +785,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="1" t="n">
-        <v>9999</v>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>900005</v>
+        <v>900011</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>20260727</v>
@@ -797,7 +805,7 @@
         <v>500005</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H8" s="1" t="n">
         <v>30717786110</v>
@@ -809,7 +817,7 @@
         <v>5747.5</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L8" s="1" t="n">
         <v>0</v>
@@ -842,13 +850,14 @@
         <v>4750</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="X8" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2"/>
       <c r="M11" s="2"/>
     </row>
   </sheetData>

</xml_diff>